<commit_message>
Work 28 Jan v3
</commit_message>
<xml_diff>
--- a/ICSummary/Dec2024/AgendaDocs/Combined-AtchisonWattle-APL.xlsx
+++ b/ICSummary/Dec2024/AgendaDocs/Combined-AtchisonWattle-APL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fa1b30dd86628461/FILE Backup/Kev/PYTHON Projects/AtchisonAnalyticsWebsite/ICSummary/Dec2024/AgendaDocs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{2C3A03DC-7CD6-40A4-8F86-DF6CD3DFB9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE14CBC0-C5F9-46CC-BB88-6B1A43070675}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{2C3A03DC-7CD6-40A4-8F86-DF6CD3DFB9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B670EAA0-86B0-4FC0-855A-4D5AF08A25D7}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3C6033BA-9EED-4A3A-A399-3C40B58B674E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3C6033BA-9EED-4A3A-A399-3C40B58B674E}"/>
   </bookViews>
   <sheets>
     <sheet name="AtchisonWattle APL" sheetId="1" r:id="rId1"/>
@@ -1974,6 +1974,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FAE6590-BB68-4477-88D7-A79F21D0D3E6}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D170"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4369,8 +4372,9 @@
     <sortCondition ref="B2:B170"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="69" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>